<commit_message>
Versi perbaikan prioritas Pertalite
</commit_message>
<xml_diff>
--- a/eksekusi.xlsx
+++ b/eksekusi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mk.irene.luarwan\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josua\Downloads\Magang_Pertamina\Project Autofill RSD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0CBA97C1-13DD-461E-8F49-A02DB27B1F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B47AEF-C175-44EA-97BD-C800B4D30B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13290" xr2:uid="{701BAB92-D1D8-4D94-B3AE-07C525A47CF0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{AB2AA2BD-83B7-40E3-80AC-BAA5AEF6EE7A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,15 +29,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="86">
   <si>
     <t>Tanggal Shipment</t>
   </si>
@@ -63,6 +60,108 @@
     <t>Segel</t>
   </si>
   <si>
+    <t>B9813SEH</t>
+  </si>
+  <si>
+    <t>FRANDY HENDRIK BORORING [73109224/1074]</t>
+  </si>
+  <si>
+    <t>8144243132,8144243126,8144243125,</t>
+  </si>
+  <si>
+    <t>BIOSOLAR B50;PERTALITE;</t>
+  </si>
+  <si>
+    <t>B9251SFW</t>
+  </si>
+  <si>
+    <t>FEBRIYANTO IS RAHMAD JAHJA [73101042]</t>
+  </si>
+  <si>
+    <t>8144244518,8144244528,</t>
+  </si>
+  <si>
+    <t>PERTALITE;</t>
+  </si>
+  <si>
+    <t>B9051SFW</t>
+  </si>
+  <si>
+    <t>HEIN RADJAK [74100114]</t>
+  </si>
+  <si>
+    <t>8144244501,8144244506,</t>
+  </si>
+  <si>
+    <t>B9050SFW</t>
+  </si>
+  <si>
+    <t>SEFRIYANTO HADJARATI [73114884]</t>
+  </si>
+  <si>
+    <t>8144244530,8144244472,</t>
+  </si>
+  <si>
+    <t>B9697SEI</t>
+  </si>
+  <si>
+    <t>FAISAL [73100120/843]</t>
+  </si>
+  <si>
+    <t>8144142722,8144142729,8144186390,</t>
+  </si>
+  <si>
+    <t>B9556SFV</t>
+  </si>
+  <si>
+    <t>FRITS TATENGKENG [73100210/84]</t>
+  </si>
+  <si>
+    <t>8144247705,8144247706,</t>
+  </si>
+  <si>
+    <t>B9536SFV</t>
+  </si>
+  <si>
+    <t>GRANDO IMANUEL KEVIN RUNTUWENE [73117379/1188]</t>
+  </si>
+  <si>
+    <t>8144241154,8143326103,8143325819,</t>
+  </si>
+  <si>
+    <t>PERTAMAX,BULK;</t>
+  </si>
+  <si>
+    <t>B9424SFV</t>
+  </si>
+  <si>
+    <t>VALENTINO PALAR [73109239/1127]</t>
+  </si>
+  <si>
+    <t>8144229026,</t>
+  </si>
+  <si>
+    <t>B9346SFV</t>
+  </si>
+  <si>
+    <t>CADAFIDNO JUSUF [73100111/842]</t>
+  </si>
+  <si>
+    <t>8144241148,8144241140,</t>
+  </si>
+  <si>
+    <t>B9636SEI</t>
+  </si>
+  <si>
+    <t>GILBERT BASSAY [73109209/1121]</t>
+  </si>
+  <si>
+    <t>8144231668,8144231667,8144231670,</t>
+  </si>
+  <si>
+    <t>PERTALITE;BIOSOLAR B50;</t>
+  </si>
+  <si>
     <t>DB8019QR</t>
   </si>
   <si>
@@ -72,9 +171,6 @@
     <t>8144229029,8144241256,8144241257,</t>
   </si>
   <si>
-    <t>PERTALITE;BIOSOLAR B50;</t>
-  </si>
-  <si>
     <t>B9689SEI</t>
   </si>
   <si>
@@ -84,7 +180,7 @@
     <t>8144143457,8144190169,8144231669,</t>
   </si>
   <si>
-    <t>PERTALITE;</t>
+    <t>1002416,1002417,1002418,1002419,1002420,1002421,</t>
   </si>
   <si>
     <t>L9757UO</t>
@@ -96,7 +192,7 @@
     <t>8144247659,8144238443,8144238440,</t>
   </si>
   <si>
-    <t>BIOSOLAR B50;PERTALITE;</t>
+    <t>1003000,1002401,1002402,1002403,1002404,1002405,</t>
   </si>
   <si>
     <t>DB8403RK</t>
@@ -147,6 +243,9 @@
     <t>PERTALITE;PERTAMAX,BULK;</t>
   </si>
   <si>
+    <t>1002412,1002413,1002414,1002415,</t>
+  </si>
+  <si>
     <t>B9149SFV</t>
   </si>
   <si>
@@ -180,6 +279,9 @@
     <t>BIOSOLAR B50;PERTAMAX,BULK;</t>
   </si>
   <si>
+    <t>1002942,1002943,1002944,1002945,1002946,1002947,</t>
+  </si>
+  <si>
     <t>B9577SEI</t>
   </si>
   <si>
@@ -189,136 +291,7 @@
     <t>8144185125,8144239717,8144239716,</t>
   </si>
   <si>
-    <t>DB8976LM</t>
-  </si>
-  <si>
-    <t>STEVEN YANCE SAWEHO [73100152/170]</t>
-  </si>
-  <si>
-    <t>8144241137,8144243149,8144241134,</t>
-  </si>
-  <si>
-    <t>1002988,1002989,1002990,1002991,1002992,1002993,</t>
-  </si>
-  <si>
-    <t>B9800SEI</t>
-  </si>
-  <si>
-    <t>MOHAMMAD ANDIKA KATILI [73100195/50]</t>
-  </si>
-  <si>
-    <t>8144229641,8144230394,8144175430,</t>
-  </si>
-  <si>
-    <t>1002958,1002959,1002960,1002961,1002962,1002963,</t>
-  </si>
-  <si>
-    <t>B9147SFV</t>
-  </si>
-  <si>
-    <t>MENLY SATRYA KARWUR [73100194/56]</t>
-  </si>
-  <si>
-    <t>8144235471,8144235472,</t>
-  </si>
-  <si>
-    <t>1002980,1002981,1002982,1002983,</t>
-  </si>
-  <si>
-    <t>B9697SEI</t>
-  </si>
-  <si>
-    <t>FAISAL [73100120/843]</t>
-  </si>
-  <si>
-    <t>8144181990,8144239725,8144239726,</t>
-  </si>
-  <si>
-    <t>1002968,1002969,1002970,1002971,1002972,1002973,</t>
-  </si>
-  <si>
-    <t>B9344SFV</t>
-  </si>
-  <si>
-    <t>ABDUL KARIM RIZAL YANTO [73118891/311]</t>
-  </si>
-  <si>
-    <t>8144241127,8144241131,</t>
-  </si>
-  <si>
-    <t>1002938,1002939,1002940,1002941,</t>
-  </si>
-  <si>
-    <t>B9598SFV</t>
-  </si>
-  <si>
-    <t>DENNY DAUD MAKALEW [73100163/1022]</t>
-  </si>
-  <si>
-    <t>8144241120,8144241121,</t>
-  </si>
-  <si>
-    <t>1002948,1002949,1002950,1002951,</t>
-  </si>
-  <si>
-    <t>B9836SFV</t>
-  </si>
-  <si>
-    <t>YUNUS PANDJU [73116567/1164]</t>
-  </si>
-  <si>
-    <t>8144233381,8144233376,</t>
-  </si>
-  <si>
-    <t>1002934,1002935,1002936,1002937,</t>
-  </si>
-  <si>
-    <t>B9257SFW</t>
-  </si>
-  <si>
-    <t>ADITYA PRASETYO LENGKONG [73109208/1119]</t>
-  </si>
-  <si>
-    <t>8144178901,8144178900,</t>
-  </si>
-  <si>
-    <t>1002964,1002965,1002966,1002967,</t>
-  </si>
-  <si>
-    <t>B9551SFV</t>
-  </si>
-  <si>
-    <t>MARSEL LAHETE [73100193/58]</t>
-  </si>
-  <si>
-    <t>8144177435,8144177431,</t>
-  </si>
-  <si>
-    <t>1002917,1002921,1002919,1002920,</t>
-  </si>
-  <si>
-    <t>B9686SEI</t>
-  </si>
-  <si>
-    <t>ISMAIL DUKALANG [73100127/850]</t>
-  </si>
-  <si>
-    <t>8144225692,8144192262,8144192255,</t>
-  </si>
-  <si>
-    <t>1002871,1002872,1002873,1002874,1002875,1002876,</t>
-  </si>
-  <si>
-    <t>B9512SFV</t>
-  </si>
-  <si>
-    <t>ALFIAN TOMPUNU [73100105/18]</t>
-  </si>
-  <si>
-    <t>8144186389,8144191134,</t>
-  </si>
-  <si>
-    <t>1002984,1002985,1002986,1002987,</t>
+    <t>1002406,1002407,1002408,1002409,1002410,1002411,</t>
   </si>
 </sst>
 </file>
@@ -670,21 +643,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A97E52D-307E-40E4-8898-F1608001AF1E}">
-  <dimension ref="A1:H43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BFD6F12-7C36-4142-A02F-CAFD9122560C}">
+  <dimension ref="A1:H53"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="30" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="47.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="47.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -710,9 +683,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>46283.444479166668</v>
+        <v>46283.520277777781</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -730,9 +703,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>46283.422615740739</v>
+        <v>46283.507037037038</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -741,7 +714,7 @@
         <v>13</v>
       </c>
       <c r="E3">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -750,9 +723,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>46283.417199074072</v>
+        <v>46283.505277777775</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
@@ -761,560 +734,549 @@
         <v>17</v>
       </c>
       <c r="E4">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
       </c>
       <c r="G4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>46283.50409722222</v>
+      </c>
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>46283.411481481482</v>
-      </c>
-      <c r="B5" s="1">
-        <v>46283.460196759261</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>20</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
         <v>21</v>
       </c>
-      <c r="E5">
-        <v>24</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>46283.495625000003</v>
+      </c>
+      <c r="C6" t="s">
         <v>22</v>
       </c>
-      <c r="G5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="D6" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>46283.390787037039</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" t="s">
-        <v>25</v>
       </c>
       <c r="E6">
         <v>24</v>
       </c>
       <c r="F6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>46283.49417824074</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
         <v>26</v>
       </c>
-      <c r="G6" t="s">
+      <c r="E7">
+        <v>16</v>
+      </c>
+      <c r="F7" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>46283.389085648145</v>
-      </c>
-      <c r="B7" s="1">
-        <v>46283.433946759258</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="G7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>46283.493680555555</v>
+      </c>
+      <c r="C8" t="s">
         <v>28</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>29</v>
       </c>
-      <c r="E7">
+      <c r="E8">
         <v>8</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F8" t="s">
         <v>30</v>
       </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="G8" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>46283.38177083333</v>
-      </c>
-      <c r="C8" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>46283.481423611112</v>
+      </c>
+      <c r="C9" t="s">
         <v>32</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D9" t="s">
         <v>33</v>
       </c>
-      <c r="E8">
-        <v>16</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9" t="s">
         <v>34</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>46283.472708333335</v>
+      </c>
+      <c r="C10" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>46283.376319444447</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="D10" t="s">
         <v>36</v>
-      </c>
-      <c r="D9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9">
-        <v>16</v>
-      </c>
-      <c r="F9" t="s">
-        <v>38</v>
-      </c>
-      <c r="G9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>46283.374513888892</v>
-      </c>
-      <c r="B10" s="1">
-        <v>46283.428090277775</v>
-      </c>
-      <c r="C10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D10" t="s">
-        <v>40</v>
       </c>
       <c r="E10">
         <v>16</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
-        <v>46283.373298611114</v>
+        <v>46283.471770833334</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E11">
         <v>24</v>
       </c>
       <c r="F11" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G11" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
-        <v>46283.366377314815</v>
+        <v>46283.444479166668</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E12">
         <v>24</v>
       </c>
       <c r="F12" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
-        <v>46283.357106481482</v>
+        <v>46283.422615740739</v>
       </c>
       <c r="B13" s="1">
-        <v>46283.45753472222</v>
+        <v>46283.486956018518</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E13">
         <v>24</v>
       </c>
       <c r="F13" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G13" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H13" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
-        <v>46283.35496527778</v>
+        <v>46283.417199074072</v>
       </c>
       <c r="B14" s="1">
-        <v>46283.421076388891</v>
+        <v>46283.471678240741</v>
       </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E14">
         <v>24</v>
       </c>
       <c r="F14" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G14" t="s">
         <v>11</v>
       </c>
       <c r="H14" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>46283.411481481482</v>
+      </c>
+      <c r="B15" s="1">
+        <v>46283.460196759261</v>
+      </c>
+      <c r="C15" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15">
+        <v>24</v>
+      </c>
+      <c r="F15" t="s">
+        <v>55</v>
+      </c>
+      <c r="G15" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>46283.390787037039</v>
+      </c>
+      <c r="C16" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
-        <v>46283.34815972222</v>
-      </c>
-      <c r="B15" s="1">
-        <v>46283.437037037038</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="D16" t="s">
         <v>58</v>
-      </c>
-      <c r="D15" t="s">
-        <v>59</v>
-      </c>
-      <c r="E15">
-        <v>16</v>
-      </c>
-      <c r="F15" t="s">
-        <v>60</v>
-      </c>
-      <c r="G15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
-        <v>46283.346608796295</v>
-      </c>
-      <c r="B16" s="1">
-        <v>46283.427777777775</v>
-      </c>
-      <c r="C16" t="s">
-        <v>62</v>
-      </c>
-      <c r="D16" t="s">
-        <v>63</v>
       </c>
       <c r="E16">
         <v>24</v>
       </c>
       <c r="F16" t="s">
+        <v>59</v>
+      </c>
+      <c r="G16" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>46283.389085648145</v>
+      </c>
+      <c r="B17" s="1">
+        <v>46283.433946759258</v>
+      </c>
+      <c r="C17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" t="s">
+        <v>62</v>
+      </c>
+      <c r="E17">
+        <v>8</v>
+      </c>
+      <c r="F17" t="s">
+        <v>63</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
         <v>64</v>
       </c>
-      <c r="G16" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" t="s">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>46283.38177083333</v>
+      </c>
+      <c r="B18" s="1">
+        <v>46283.481840277775</v>
+      </c>
+      <c r="C18" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <v>46283.341678240744</v>
-      </c>
-      <c r="B17" s="1">
-        <v>46283.390740740739</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="D18" t="s">
         <v>66</v>
-      </c>
-      <c r="D17" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17">
-        <v>16</v>
-      </c>
-      <c r="F17" t="s">
-        <v>68</v>
-      </c>
-      <c r="G17" t="s">
-        <v>11</v>
-      </c>
-      <c r="H17" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>46283.334537037037</v>
-      </c>
-      <c r="B18" s="1">
-        <v>46283.397800925923</v>
-      </c>
-      <c r="C18" t="s">
-        <v>70</v>
-      </c>
-      <c r="D18" t="s">
-        <v>71</v>
       </c>
       <c r="E18">
         <v>16</v>
       </c>
       <c r="F18" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="G18" t="s">
-        <v>15</v>
+        <v>68</v>
       </c>
       <c r="H18" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
-        <v>46283.333287037036</v>
-      </c>
-      <c r="B19" s="1">
-        <v>46283.378252314818</v>
+        <v>46283.376319444447</v>
       </c>
       <c r="C19" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D19" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E19">
         <v>16</v>
       </c>
       <c r="F19" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G19" t="s">
-        <v>19</v>
-      </c>
-      <c r="H19" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
-        <v>46283.332442129627</v>
+        <v>46283.374513888892</v>
       </c>
       <c r="B20" s="1">
-        <v>46283.418275462966</v>
+        <v>46283.428090277775</v>
       </c>
       <c r="C20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E20">
         <v>16</v>
       </c>
       <c r="F20" t="s">
+        <v>75</v>
+      </c>
+      <c r="G20" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>46283.373298611114</v>
+      </c>
+      <c r="B21" s="1">
+        <v>46283.470127314817</v>
+      </c>
+      <c r="C21" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E21">
+        <v>24</v>
+      </c>
+      <c r="F21" t="s">
+        <v>79</v>
+      </c>
+      <c r="G21" t="s">
         <v>80</v>
       </c>
-      <c r="G20" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="H21" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>46283.330578703702</v>
-      </c>
-      <c r="B21" s="1">
-        <v>46283.35728009259</v>
-      </c>
-      <c r="C21" t="s">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>46283.366377314815</v>
+      </c>
+      <c r="B22" s="1">
+        <v>46283.481006944443</v>
+      </c>
+      <c r="C22" t="s">
         <v>82</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D22" t="s">
         <v>83</v>
-      </c>
-      <c r="E21">
-        <v>16</v>
-      </c>
-      <c r="F21" t="s">
-        <v>84</v>
-      </c>
-      <c r="G21" t="s">
-        <v>19</v>
-      </c>
-      <c r="H21" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <v>46283.324606481481</v>
-      </c>
-      <c r="B22" s="1">
-        <v>46283.326192129629</v>
-      </c>
-      <c r="C22" t="s">
-        <v>86</v>
-      </c>
-      <c r="D22" t="s">
-        <v>87</v>
       </c>
       <c r="E22">
         <v>24</v>
       </c>
       <c r="F22" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G22" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="H22" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
-        <v>46283.29991898148</v>
-      </c>
-      <c r="B27" s="1">
-        <v>46283.445520833331</v>
-      </c>
-      <c r="C27" t="s">
-        <v>90</v>
-      </c>
-      <c r="D27" t="s">
-        <v>91</v>
-      </c>
-      <c r="E27">
-        <v>16</v>
-      </c>
-      <c r="F27" t="s">
-        <v>92</v>
-      </c>
-      <c r="G27" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
     </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="1"/>
+      <c r="B44" s="1"/>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" s="1"/>
+      <c r="B45" s="1"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" s="1"/>
+      <c r="B46" s="1"/>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" s="1"/>
+      <c r="B47" s="1"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="1"/>
+      <c r="B48" s="1"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="1"/>
+      <c r="B49" s="1"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="1"/>
+      <c r="B50" s="1"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="1"/>
+      <c r="B51" s="1"/>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="1"/>
+      <c r="B52" s="1"/>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="1"/>
+      <c r="B53" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Versi Stabil Autofill SNDone
</commit_message>
<xml_diff>
--- a/eksekusi.xlsx
+++ b/eksekusi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josua\Downloads\Magang_Pertamina\Project Autofill RSD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mk.irene.luarwan\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B47AEF-C175-44EA-97BD-C800B4D30B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{133D1118-E6DA-457F-979D-659E94DCC98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{AB2AA2BD-83B7-40E3-80AC-BAA5AEF6EE7A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13290" xr2:uid="{87218AE3-D482-4D59-AC6C-EA15ADC6F476}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="85">
   <si>
     <t>Tanggal Shipment</t>
   </si>
@@ -60,106 +63,112 @@
     <t>Segel</t>
   </si>
   <si>
-    <t>B9813SEH</t>
-  </si>
-  <si>
-    <t>FRANDY HENDRIK BORORING [73109224/1074]</t>
-  </si>
-  <si>
-    <t>8144243132,8144243126,8144243125,</t>
+    <t>B9956SFV</t>
+  </si>
+  <si>
+    <t>STEVANO KURNIA TUMBEL [73109238/1126]</t>
+  </si>
+  <si>
+    <t>8144505882,8144505054,</t>
+  </si>
+  <si>
+    <t>PERTALITE;</t>
+  </si>
+  <si>
+    <t>B9689SEI</t>
+  </si>
+  <si>
+    <t>REVANO SEMUEL LINTANG [4688-32/1137]</t>
+  </si>
+  <si>
+    <t>8144486906,8144486905,8144486908,</t>
+  </si>
+  <si>
+    <t>PERTALITE;BIOSOLAR B50;</t>
+  </si>
+  <si>
+    <t>B9636SEI</t>
+  </si>
+  <si>
+    <t>GILBERT BASSAY [73109209/1121]</t>
+  </si>
+  <si>
+    <t>8144414274,8144460680,8144487145,</t>
+  </si>
+  <si>
+    <t>B9291SFV</t>
+  </si>
+  <si>
+    <t>VICKY JULIMAN HALEAN [73109198/1086]</t>
+  </si>
+  <si>
+    <t>8144460684,8144505896,</t>
+  </si>
+  <si>
+    <t>B9551SFV</t>
+  </si>
+  <si>
+    <t>ABDUL KARIM RIZAL YANTO [73118891/311]</t>
+  </si>
+  <si>
+    <t>8144397424,8144499028,</t>
+  </si>
+  <si>
+    <t>L9757UO</t>
+  </si>
+  <si>
+    <t>CANSTEEL RICHARD KOLIBU [73109192/1071]</t>
+  </si>
+  <si>
+    <t>8144499438,8144508497,8144499436,</t>
+  </si>
+  <si>
+    <t>B9726SFU</t>
+  </si>
+  <si>
+    <t>CANDRA NOVI LASUT [73100188/46]</t>
+  </si>
+  <si>
+    <t>8144414284,8144504370,</t>
+  </si>
+  <si>
+    <t>PERTALITE;DEXLITE;</t>
+  </si>
+  <si>
+    <t>B9630SEI</t>
+  </si>
+  <si>
+    <t>MAICHEL SILVANUS MANIS [73109236/1124]</t>
+  </si>
+  <si>
+    <t>8144503660,8144503651,8144503661,</t>
+  </si>
+  <si>
+    <t>111158,111159,111160,111161,111162,111163,</t>
+  </si>
+  <si>
+    <t>B9882SFV</t>
+  </si>
+  <si>
+    <t>GUSTIBUS IRALA [73100259/1038]</t>
+  </si>
+  <si>
+    <t>8144494607,8144492712,</t>
   </si>
   <si>
     <t>BIOSOLAR B50;PERTALITE;</t>
   </si>
   <si>
-    <t>B9251SFW</t>
-  </si>
-  <si>
-    <t>FEBRIYANTO IS RAHMAD JAHJA [73101042]</t>
-  </si>
-  <si>
-    <t>8144244518,8144244528,</t>
-  </si>
-  <si>
-    <t>PERTALITE;</t>
-  </si>
-  <si>
-    <t>B9051SFW</t>
-  </si>
-  <si>
-    <t>HEIN RADJAK [74100114]</t>
-  </si>
-  <si>
-    <t>8144244501,8144244506,</t>
-  </si>
-  <si>
-    <t>B9050SFW</t>
-  </si>
-  <si>
-    <t>SEFRIYANTO HADJARATI [73114884]</t>
-  </si>
-  <si>
-    <t>8144244530,8144244472,</t>
-  </si>
-  <si>
-    <t>B9697SEI</t>
-  </si>
-  <si>
-    <t>FAISAL [73100120/843]</t>
-  </si>
-  <si>
-    <t>8144142722,8144142729,8144186390,</t>
-  </si>
-  <si>
-    <t>B9556SFV</t>
-  </si>
-  <si>
-    <t>FRITS TATENGKENG [73100210/84]</t>
-  </si>
-  <si>
-    <t>8144247705,8144247706,</t>
-  </si>
-  <si>
-    <t>B9536SFV</t>
-  </si>
-  <si>
-    <t>GRANDO IMANUEL KEVIN RUNTUWENE [73117379/1188]</t>
-  </si>
-  <si>
-    <t>8144241154,8143326103,8143325819,</t>
-  </si>
-  <si>
-    <t>PERTAMAX,BULK;</t>
-  </si>
-  <si>
-    <t>B9424SFV</t>
-  </si>
-  <si>
-    <t>VALENTINO PALAR [73109239/1127]</t>
-  </si>
-  <si>
-    <t>8144229026,</t>
-  </si>
-  <si>
-    <t>B9346SFV</t>
-  </si>
-  <si>
-    <t>CADAFIDNO JUSUF [73100111/842]</t>
-  </si>
-  <si>
-    <t>8144241148,8144241140,</t>
-  </si>
-  <si>
-    <t>B9636SEI</t>
-  </si>
-  <si>
-    <t>GILBERT BASSAY [73109209/1121]</t>
-  </si>
-  <si>
-    <t>8144231668,8144231667,8144231670,</t>
-  </si>
-  <si>
-    <t>PERTALITE;BIOSOLAR B50;</t>
+    <t>111200,1016801,1016802,1016803,</t>
+  </si>
+  <si>
+    <t>DB8015RK</t>
+  </si>
+  <si>
+    <t>DEVI LENGKEY [73100116/118]</t>
+  </si>
+  <si>
+    <t>8144489488,8144500767,8144499443,</t>
   </si>
   <si>
     <t>DB8019QR</t>
@@ -168,130 +177,121 @@
     <t>FAHRIL ABDULLAH [73109223/1073]</t>
   </si>
   <si>
-    <t>8144229029,8144241256,8144241257,</t>
-  </si>
-  <si>
-    <t>B9689SEI</t>
-  </si>
-  <si>
-    <t>MESAK SASIKOME [73100213/78]</t>
-  </si>
-  <si>
-    <t>8144143457,8144190169,8144231669,</t>
-  </si>
-  <si>
-    <t>1002416,1002417,1002418,1002419,1002420,1002421,</t>
-  </si>
-  <si>
-    <t>L9757UO</t>
-  </si>
-  <si>
-    <t>CANSTEEL RICHARD KOLIBU [73109192/1071]</t>
-  </si>
-  <si>
-    <t>8144247659,8144238443,8144238440,</t>
-  </si>
-  <si>
-    <t>1003000,1002401,1002402,1002403,1002404,1002405,</t>
+    <t>8144505893,8144505895,8144502800,</t>
+  </si>
+  <si>
+    <t>111178,111179,111180,111181,111182,111183,</t>
   </si>
   <si>
     <t>DB8403RK</t>
   </si>
   <si>
-    <t>RENALDI MELKI SUMANGANDO [73100176/162]</t>
-  </si>
-  <si>
-    <t>8144250653,8144250654,8144250649,</t>
-  </si>
-  <si>
-    <t>1002994,1002995,1002996,1002997,1002998,1002999,</t>
-  </si>
-  <si>
-    <t>DB8015RK</t>
-  </si>
-  <si>
-    <t>KRIS VIERI JULIAN SINERI [73118933/3006]</t>
-  </si>
-  <si>
-    <t>8144243120,8144190155,8144243123,</t>
-  </si>
-  <si>
-    <t>PERTAMAX,BULK;PERTALITE;</t>
+    <t>BRIAN ADAM MAHULETE [73100243/1101]</t>
+  </si>
+  <si>
+    <t>8144510817,8144510816,8144509361,</t>
+  </si>
+  <si>
+    <t>PERTALITE;PERTAMAX,BULK;</t>
+  </si>
+  <si>
+    <t>111184,111185,111186,111187,111188,111189,</t>
+  </si>
+  <si>
+    <t>B9270SFW</t>
+  </si>
+  <si>
+    <t>DANISA ROMPAS [73116583/1170]</t>
+  </si>
+  <si>
+    <t>8144501293,8144501299,</t>
+  </si>
+  <si>
+    <t>111174,111175,111176,111177,</t>
+  </si>
+  <si>
+    <t>DB8976LM</t>
+  </si>
+  <si>
+    <t>EKO RIZKY HEIN AWALI [73109230/1097]</t>
+  </si>
+  <si>
+    <t>8144512021,8144512025,8144512022,</t>
+  </si>
+  <si>
+    <t>111168,111169,111170,111171,111172,111173,</t>
+  </si>
+  <si>
+    <t>DB8016RK</t>
+  </si>
+  <si>
+    <t>DENDY REYFORD TULAR [73100220/91]</t>
+  </si>
+  <si>
+    <t>8144486898,8144486899,8144486903,</t>
+  </si>
+  <si>
+    <t>111148,111149,111150,111151,111152,111153,</t>
+  </si>
+  <si>
+    <t>B9257SFW</t>
+  </si>
+  <si>
+    <t>ADITYA PRASETYO LENGKONG [73109208/1119]</t>
+  </si>
+  <si>
+    <t>8144492103,8144494603,</t>
+  </si>
+  <si>
+    <t>111164,111165,111166,111167,</t>
+  </si>
+  <si>
+    <t>B9836SFV</t>
+  </si>
+  <si>
+    <t>YUNUS PANDJU [73116567/1164]</t>
+  </si>
+  <si>
+    <t>8144487142,8144487143,</t>
+  </si>
+  <si>
+    <t>111144,111145,111146,111147,</t>
+  </si>
+  <si>
+    <t>B9149SFV</t>
+  </si>
+  <si>
+    <t>CARLOS GEOVANI SANDEHANG [73109193/1072]</t>
+  </si>
+  <si>
+    <t>8144502769,8144466067,</t>
+  </si>
+  <si>
+    <t>111140,111141,111142,111143,</t>
   </si>
   <si>
     <t>B9408SFV</t>
   </si>
   <si>
-    <t>JENER OVER PUDI [73117102/1186]</t>
-  </si>
-  <si>
-    <t>8144249391,</t>
-  </si>
-  <si>
-    <t>1002978,1002979,</t>
-  </si>
-  <si>
-    <t>B9291SFV</t>
-  </si>
-  <si>
-    <t>VICKY JULIMAN HALEAN [73109198/1086]</t>
-  </si>
-  <si>
-    <t>8144245330,8144244778,</t>
-  </si>
-  <si>
-    <t>PERTALITE;PERTAMAX,BULK;</t>
-  </si>
-  <si>
-    <t>1002412,1002413,1002414,1002415,</t>
-  </si>
-  <si>
-    <t>B9149SFV</t>
-  </si>
-  <si>
-    <t>CHRISTIAN FERNANDES TAROREH [73100250/1024]</t>
-  </si>
-  <si>
-    <t>8144239750,8144239752,</t>
-  </si>
-  <si>
-    <t>B9882SFV</t>
-  </si>
-  <si>
-    <t>GUSTIBUS IRALA [73100259/1038]</t>
-  </si>
-  <si>
-    <t>8144230825,8144230821,</t>
-  </si>
-  <si>
-    <t>1002974,1002975,1002976,1002977,</t>
-  </si>
-  <si>
-    <t>B9630SEI</t>
-  </si>
-  <si>
-    <t>ANDRE RARAMENUSA TILAAR [73100249/1031]</t>
-  </si>
-  <si>
-    <t>8144181996,8144239731,8144239733,</t>
-  </si>
-  <si>
-    <t>BIOSOLAR B50;PERTAMAX,BULK;</t>
-  </si>
-  <si>
-    <t>1002942,1002943,1002944,1002945,1002946,1002947,</t>
-  </si>
-  <si>
-    <t>B9577SEI</t>
-  </si>
-  <si>
-    <t>JULIO AQBAR KOMALIG [73100235/113]</t>
-  </si>
-  <si>
-    <t>8144185125,8144239717,8144239716,</t>
-  </si>
-  <si>
-    <t>1002406,1002407,1002408,1002409,1002410,1002411,</t>
+    <t>ERWIN ARIEF [73100119/123]</t>
+  </si>
+  <si>
+    <t>8144509310,</t>
+  </si>
+  <si>
+    <t>111138,111139,</t>
+  </si>
+  <si>
+    <t>B9147SFV</t>
+  </si>
+  <si>
+    <t>BILLY AGUNG LINTJEWAS [73117382/1199]</t>
+  </si>
+  <si>
+    <t>8144488533,8144488534,</t>
+  </si>
+  <si>
+    <t>111154,111155,111156,111157,</t>
   </si>
 </sst>
 </file>
@@ -327,9 +327,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -643,21 +644,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BFD6F12-7C36-4142-A02F-CAFD9122560C}">
-  <dimension ref="A1:H53"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD0FB8CC-3E30-4D1C-923A-FD34C46AFB72}">
+  <dimension ref="A1:H48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="51.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="47.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="44.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="41.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -683,9 +684,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>46283.520277777781</v>
+        <v>46289.440555555557</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -694,7 +695,7 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -703,9 +704,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>46283.507037037038</v>
+        <v>46289.427928240744</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -714,7 +715,7 @@
         <v>13</v>
       </c>
       <c r="E3">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -723,9 +724,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>46283.505277777775</v>
+        <v>46289.427476851852</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
@@ -734,18 +735,18 @@
         <v>17</v>
       </c>
       <c r="E4">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>46283.50409722222</v>
+        <v>46289.40898148148</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -760,12 +761,12 @@
         <v>21</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>46283.495625000003</v>
+        <v>46289.408634259256</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -774,18 +775,18 @@
         <v>23</v>
       </c>
       <c r="E6">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F6" t="s">
         <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>46283.49417824074</v>
+        <v>46289.402754629627</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
@@ -794,18 +795,18 @@
         <v>26</v>
       </c>
       <c r="E7">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F7" t="s">
         <v>27</v>
       </c>
       <c r="G7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>46283.493680555555</v>
+        <v>46289.402106481481</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -814,7 +815,7 @@
         <v>29</v>
       </c>
       <c r="E8">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F8" t="s">
         <v>30</v>
@@ -823,9 +824,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>46283.481423611112</v>
+        <v>46289.385636574072</v>
+      </c>
+      <c r="B9" s="2">
+        <v>46289.444319340277</v>
       </c>
       <c r="C9" t="s">
         <v>32</v>
@@ -834,449 +838,433 @@
         <v>33</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="F9" t="s">
         <v>34</v>
       </c>
       <c r="G9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>46283.472708333335</v>
+        <v>46289.383472222224</v>
+      </c>
+      <c r="B10" s="1">
+        <v>46289.441516203704</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E10">
         <v>16</v>
       </c>
       <c r="F10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="H10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>46283.471770833334</v>
+        <v>46289.383194444446</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E11">
         <v>24</v>
       </c>
       <c r="F11" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>46283.444479166668</v>
+        <v>46289.378912037035</v>
+      </c>
+      <c r="B12" s="1">
+        <v>46289.427905092591</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E12">
         <v>24</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G12" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>46283.422615740739</v>
+        <v>46289.373831018522</v>
       </c>
       <c r="B13" s="1">
-        <v>46283.486956018518</v>
+        <v>46289.428518518522</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D13" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E13">
         <v>24</v>
       </c>
       <c r="F13" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G13" t="s">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="H13" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>46283.417199074072</v>
+        <v>46289.372696759259</v>
       </c>
       <c r="B14" s="1">
-        <v>46283.471678240741</v>
+        <v>46289.417870370373</v>
       </c>
       <c r="C14" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D14" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E14">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G14" t="s">
         <v>11</v>
       </c>
       <c r="H14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>46283.411481481482</v>
+        <v>46289.367777777778</v>
       </c>
       <c r="B15" s="1">
-        <v>46283.460196759261</v>
+        <v>46289.417199074072</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E15">
         <v>24</v>
       </c>
       <c r="F15" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G15" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="H15" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>46283.390787037039</v>
+        <v>46289.350277777776</v>
+      </c>
+      <c r="B16" s="1">
+        <v>46289.38894675926</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D16" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E16">
         <v>24</v>
       </c>
       <c r="F16" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G16" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>46283.389085648145</v>
+        <v>46289.349791666667</v>
       </c>
       <c r="B17" s="1">
-        <v>46283.433946759258</v>
+        <v>46289.408402777779</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D17" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E17">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F17" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G17" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H17" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>46283.38177083333</v>
+        <v>46289.343923611108</v>
       </c>
       <c r="B18" s="1">
-        <v>46283.481840277775</v>
+        <v>46289.388622685183</v>
       </c>
       <c r="C18" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="E18">
         <v>16</v>
       </c>
       <c r="F18" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G18" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="H18" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>46283.376319444447</v>
+        <v>46289.343692129631</v>
+      </c>
+      <c r="B19" s="1">
+        <v>46289.379756944443</v>
       </c>
       <c r="C19" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E19">
         <v>16</v>
       </c>
       <c r="F19" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G19" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>46283.374513888892</v>
+        <v>46289.341805555552</v>
       </c>
       <c r="B20" s="1">
-        <v>46283.428090277775</v>
+        <v>46289.378831018519</v>
       </c>
       <c r="C20" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D20" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E20">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G20" t="s">
         <v>11</v>
       </c>
       <c r="H20" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>46283.373298611114</v>
+        <v>46289.317986111113</v>
       </c>
       <c r="B21" s="1">
-        <v>46283.470127314817</v>
+        <v>46289.389791666668</v>
       </c>
       <c r="C21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E21">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F21" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G21" t="s">
-        <v>80</v>
+        <v>11</v>
       </c>
       <c r="H21" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="1">
-        <v>46283.366377314815</v>
-      </c>
-      <c r="B22" s="1">
-        <v>46283.481006944443</v>
-      </c>
-      <c r="C22" t="s">
-        <v>82</v>
-      </c>
-      <c r="D22" t="s">
-        <v>83</v>
-      </c>
-      <c r="E22">
-        <v>24</v>
-      </c>
-      <c r="F22" t="s">
         <v>84</v>
       </c>
-      <c r="G22" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="1"/>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B37" s="2"/>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
-      <c r="B42" s="1"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B42" s="2"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="1"/>
-      <c r="B50" s="1"/>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" s="1"/>
-      <c r="B52" s="1"/>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" s="1"/>
-      <c r="B53" s="1"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Autofill Versi penyesuaian blank nopol
</commit_message>
<xml_diff>
--- a/eksekusi.xlsx
+++ b/eksekusi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mk.irene.luarwan\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4888E870-D81D-4BB5-A26F-3B44DA67C995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{661F799C-16D8-49AD-87F9-0D96FD4B656F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13290" xr2:uid="{A1A51837-6E48-4DEB-84CA-48F618AB177D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13290" xr2:uid="{2E946F75-FCC6-4324-8BF0-1B2AA243E1F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="127">
   <si>
     <t>Tanggal Shipment</t>
   </si>
@@ -63,73 +63,361 @@
     <t>Segel</t>
   </si>
   <si>
+    <t>B9630SEI</t>
+  </si>
+  <si>
+    <t>ANDRE RARAMENUSA TILAAR [73100249/1031]</t>
+  </si>
+  <si>
+    <t>8144751703,8144751704,8144751707,</t>
+  </si>
+  <si>
+    <t>PERTALITE;BIOSOLAR B50;</t>
+  </si>
+  <si>
+    <t>B9344SFV</t>
+  </si>
+  <si>
+    <t>ERICK OKTAVIAN KARUNDENG [73100165/838]</t>
+  </si>
+  <si>
+    <t>8144797881,8144757628,</t>
+  </si>
+  <si>
+    <t>PERTALITE;</t>
+  </si>
+  <si>
+    <t>B9956SFV</t>
+  </si>
+  <si>
+    <t>Kiven Kigend Rivaldo Randang [73114560/1142]</t>
+  </si>
+  <si>
+    <t>8144800992,8144800995,</t>
+  </si>
+  <si>
+    <t>B9598SFV</t>
+  </si>
+  <si>
+    <t>DENNY DAUD MAKALEW [73100163/1022]</t>
+  </si>
+  <si>
+    <t>8144781586,8144781584,</t>
+  </si>
+  <si>
+    <t>DB8976LM</t>
+  </si>
+  <si>
+    <t>FAISAL [73100120/843]</t>
+  </si>
+  <si>
+    <t>8144797874,8144780932,8144780931,</t>
+  </si>
+  <si>
+    <t>B9551SFV</t>
+  </si>
+  <si>
+    <t>THOMAS YANDRI KAUNANG [73109220/1065]</t>
+  </si>
+  <si>
+    <t>8144785820,8144804023,</t>
+  </si>
+  <si>
+    <t>B9697SEI</t>
+  </si>
+  <si>
+    <t>NOVRI LAHENGKO [73100140/845]</t>
+  </si>
+  <si>
+    <t>8144756185,8144756191,8144791355,</t>
+  </si>
+  <si>
+    <t>BIOSOLAR B50;PERTALITE;</t>
+  </si>
+  <si>
+    <t>B9464SFV</t>
+  </si>
+  <si>
+    <t>YULIO SUMENDONG [73109194/1080]</t>
+  </si>
+  <si>
+    <t>8144805819,8144805807,</t>
+  </si>
+  <si>
+    <t>B9147SFV</t>
+  </si>
+  <si>
+    <t>YANTO SUTRISNO AKUMI [73100157/835]</t>
+  </si>
+  <si>
+    <t>8144801007,8144801010,</t>
+  </si>
+  <si>
+    <t>B9577SEI</t>
+  </si>
+  <si>
+    <t>JULIO AQBAR KOMALIG [73100235/113]</t>
+  </si>
+  <si>
+    <t>8144797861,8144790786,8144790787,</t>
+  </si>
+  <si>
+    <t>1005707,1005708,1005709,1005710,1005711,1005712,</t>
+  </si>
+  <si>
+    <t>B9255SFW</t>
+  </si>
+  <si>
+    <t>ARTHER AGUSTINUS RAWA [73100110/106]</t>
+  </si>
+  <si>
+    <t>8144780175,8144789233,</t>
+  </si>
+  <si>
+    <t>L9757UO</t>
+  </si>
+  <si>
+    <t>AHMAD RIJAL TOWOLIU [73100159/889]</t>
+  </si>
+  <si>
+    <t>8144789649,8144711448,8144783483,</t>
+  </si>
+  <si>
+    <t>B9897SFV</t>
+  </si>
+  <si>
+    <t>BUDI SAPUTRA CHALIM [73109229/1095]</t>
+  </si>
+  <si>
+    <t>8144810966,8144807413,</t>
+  </si>
+  <si>
+    <t>1005691,1005692,1005693,1005694,</t>
+  </si>
+  <si>
+    <t>DB8403RK</t>
+  </si>
+  <si>
+    <t>KRIS VIERI JULIAN SINERI [73118933/3006]</t>
+  </si>
+  <si>
+    <t>8144751695,8144751696,8144751698,</t>
+  </si>
+  <si>
+    <t>1005701,1005702,1005703,1005704,1005705,1005706,</t>
+  </si>
+  <si>
+    <t>B9824SFU</t>
+  </si>
+  <si>
+    <t>Luis Fernando Sidangoli [73116110/1147]</t>
+  </si>
+  <si>
+    <t>8144797893,8144797894,</t>
+  </si>
+  <si>
+    <t>1005687,1005688,1005689,1005690,</t>
+  </si>
+  <si>
+    <t>B9251SFW</t>
+  </si>
+  <si>
+    <t>FANLY S ISMAIL [73114890/9874]</t>
+  </si>
+  <si>
+    <t>8144804817,8144804909,</t>
+  </si>
+  <si>
+    <t>DEXLITE;</t>
+  </si>
+  <si>
+    <t>1005667,1005668,1005669,1005670,</t>
+  </si>
+  <si>
+    <t>B9720SFV</t>
+  </si>
+  <si>
+    <t>FRITS TATENGKENG [73100210/84]</t>
+  </si>
+  <si>
+    <t>8144781568,8144779613,</t>
+  </si>
+  <si>
+    <t>PERTALITE;PERTAMAX,BULK;</t>
+  </si>
+  <si>
+    <t>1005673,1005674,1005675,1005676,</t>
+  </si>
+  <si>
+    <t>B9636SEI</t>
+  </si>
+  <si>
+    <t>MARVIL BRYAN OCTAVIANUS GOSAL [73116565/1163]</t>
+  </si>
+  <si>
+    <t>8144720047,8144756189,8144756190,</t>
+  </si>
+  <si>
+    <t>1005695,1005696,1005697,1005698,1005699,1005700,</t>
+  </si>
+  <si>
+    <t>B9882SFV</t>
+  </si>
+  <si>
+    <t>RENAL LANGUJU [73100198/54]</t>
+  </si>
+  <si>
+    <t>8144804017,8144789237,</t>
+  </si>
+  <si>
+    <t>BIOSOLAR B50;</t>
+  </si>
+  <si>
+    <t>1005640,1005641,1005642,1005643,</t>
+  </si>
+  <si>
+    <t>B9408SFV</t>
+  </si>
+  <si>
+    <t>JUN RICHMIN SAMBENAUNG [73119375/324]</t>
+  </si>
+  <si>
+    <t>8144811972,</t>
+  </si>
+  <si>
+    <t>1005671,1005672,</t>
+  </si>
+  <si>
+    <t>B9536SFV</t>
+  </si>
+  <si>
+    <t>CHRISTIAN MALDINI NATARANG [73118910/4321]</t>
+  </si>
+  <si>
+    <t>8144793969,</t>
+  </si>
+  <si>
+    <t>1005654,1005655,1005656,</t>
+  </si>
+  <si>
+    <t>B9686SFV</t>
+  </si>
+  <si>
+    <t>HEROL SANGGELE [73100227/1007]</t>
+  </si>
+  <si>
+    <t>8144763326,8144791338,</t>
+  </si>
+  <si>
+    <t>1005644,1005645,1005646,1005647,</t>
+  </si>
+  <si>
+    <t>B9899SFU</t>
+  </si>
+  <si>
+    <t>MAHARDIKA LESMANA [73100254/1028]</t>
+  </si>
+  <si>
+    <t>8144805894,8144800466,</t>
+  </si>
+  <si>
+    <t>1005677,1005678,1005679,1005680,</t>
+  </si>
+  <si>
+    <t>DB8019QR</t>
+  </si>
+  <si>
+    <t>RAHMAN NUR [73100144/818]</t>
+  </si>
+  <si>
+    <t>8144672945,8144805890,8144711499,</t>
+  </si>
+  <si>
+    <t>1005648,1005649,1005650,1005651,1005652,1005653,</t>
+  </si>
+  <si>
+    <t>L9963UB</t>
+  </si>
+  <si>
+    <t>FELIX RONALD WONGKAR [SINTUWU-002/796]</t>
+  </si>
+  <si>
+    <t>8144802197,8144802170,8144802171,</t>
+  </si>
+  <si>
+    <t>1005681,1005682,1005683,1005684,1005685,1005686,</t>
+  </si>
+  <si>
+    <t>B9543SFV</t>
+  </si>
+  <si>
+    <t>SUCIPTO ANWAR TALIB [73100199/196]</t>
+  </si>
+  <si>
+    <t>8144763322,8144763323,</t>
+  </si>
+  <si>
+    <t>1005663,1005664,1005665,1005666,</t>
+  </si>
+  <si>
+    <t>DB8016RK</t>
+  </si>
+  <si>
+    <t>ALFREY ROMPAH [73100236/905]</t>
+  </si>
+  <si>
+    <t>8144805853,8144805829,8144805828,</t>
+  </si>
+  <si>
+    <t>1005657,1005658,1005659,1005660,1005661,1005662,</t>
+  </si>
+  <si>
+    <t>B9956SFU</t>
+  </si>
+  <si>
+    <t>MIRSAL ARIFIN [73109216/1060]</t>
+  </si>
+  <si>
+    <t>8144791343,8144791344,</t>
+  </si>
+  <si>
+    <t>1005632,1005633,1005634,1005635,</t>
+  </si>
+  <si>
+    <t>B9257SFW</t>
+  </si>
+  <si>
+    <t>DECKY OCTAVIAN KONENG [73118892/3004]</t>
+  </si>
+  <si>
+    <t>8144802179,8144801001,</t>
+  </si>
+  <si>
+    <t>1005628,1005629,1005630,1005631,</t>
+  </si>
+  <si>
+    <t>DB8017RK</t>
+  </si>
+  <si>
+    <t>AMSAL MATEDE [73100107/1018]</t>
+  </si>
+  <si>
+    <t>8144808395,8144799238,8144799239,</t>
+  </si>
+  <si>
+    <t>1005618,1005619,1005620,1005621,1005622,1005623,</t>
+  </si>
+  <si>
     <t>B9149SFV</t>
   </si>
   <si>
     <t>AMSUN LAKORU [73100108/1013]</t>
   </si>
   <si>
-    <t>8144665538,8144665539,</t>
-  </si>
-  <si>
-    <t>PERTALITE;</t>
-  </si>
-  <si>
-    <t>B9882SFV</t>
-  </si>
-  <si>
-    <t>RENAL LANGUJU [73100198/54]</t>
-  </si>
-  <si>
-    <t>8144671049,8144587680,</t>
-  </si>
-  <si>
-    <t>BIOSOLAR B50;PERTALITE;</t>
-  </si>
-  <si>
-    <t>B9408SFV</t>
-  </si>
-  <si>
-    <t>BELDI ANDREAS TANGKILISAN [73116580/1184]</t>
-  </si>
-  <si>
-    <t>8144601928,</t>
-  </si>
-  <si>
-    <t>B9815SEH</t>
-  </si>
-  <si>
-    <t>DANNY DAVID MANGINDAAN [73100113/856]</t>
-  </si>
-  <si>
-    <t>8144655089,8144655087,8144655092,</t>
-  </si>
-  <si>
-    <t>114443,114444,114445,114446,114447,114448,</t>
-  </si>
-  <si>
-    <t>B9147SFV</t>
-  </si>
-  <si>
-    <t>YANTO SUTRISNO AKUMI [73100157/835]</t>
-  </si>
-  <si>
-    <t>8144676386,8144673732,</t>
-  </si>
-  <si>
-    <t>114439,114440,114441,114442,</t>
-  </si>
-  <si>
-    <t>B9577SEI</t>
-  </si>
-  <si>
-    <t>JULIO AQBAR KOMALIG [73100235/113]</t>
-  </si>
-  <si>
-    <t>8144655465,8144674511,8144671900,</t>
-  </si>
-  <si>
-    <t>114433,114434,114435,114436,114437,114438,</t>
+    <t>8144781838,8144781840,</t>
+  </si>
+  <si>
+    <t>1005636,1005637,1005638,1005639,</t>
   </si>
 </sst>
 </file>
@@ -165,10 +453,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -482,8 +769,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22D69A59-EA68-4B58-A595-05389AE7A2E5}">
-  <dimension ref="A1:H60"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD7C3A03-444B-47BB-AE5D-65F2652BB32F}">
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
@@ -493,7 +780,7 @@
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="47.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -524,7 +811,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>46293.608807870369</v>
+        <v>46296.422199074077</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -533,7 +820,7 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -544,7 +831,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>46293.608159722222</v>
+        <v>46296.412511574075</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -564,7 +851,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>46293.603078703702</v>
+        <v>46296.409733796296</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
@@ -573,21 +860,18 @@
         <v>17</v>
       </c>
       <c r="E4">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>46293.602326388886</v>
-      </c>
-      <c r="B5" s="1">
-        <v>46293.603854166664</v>
+        <v>46296.406736111108</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -596,169 +880,674 @@
         <v>20</v>
       </c>
       <c r="E5">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s">
         <v>21</v>
       </c>
       <c r="G5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>46293.568657407406</v>
-      </c>
-      <c r="B6" s="1">
-        <v>46293.597372685188</v>
+        <v>46296.400717592594</v>
       </c>
       <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6">
         <v>24</v>
       </c>
-      <c r="E6">
-        <v>16</v>
-      </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>46293.565717592595</v>
-      </c>
-      <c r="B7" s="2">
-        <v>46293.607921168979</v>
+        <v>46296.396319444444</v>
       </c>
       <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7">
+        <v>16</v>
+      </c>
+      <c r="F7" t="s">
         <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7">
-        <v>24</v>
-      </c>
-      <c r="F7" t="s">
-        <v>29</v>
       </c>
       <c r="G7" t="s">
         <v>15</v>
       </c>
-      <c r="H7" t="s">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>46296.393958333334</v>
+      </c>
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8">
+        <v>24</v>
+      </c>
+      <c r="F8" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
+      <c r="G8" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
+      <c r="A9" s="1">
+        <v>46296.381597222222</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9">
+        <v>16</v>
+      </c>
+      <c r="F9" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
+      <c r="A10" s="1">
+        <v>46296.371979166666</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10">
+        <v>16</v>
+      </c>
+      <c r="F10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
+      <c r="A11" s="1">
+        <v>46296.352106481485</v>
+      </c>
+      <c r="B11" s="1">
+        <v>46296.413900462961</v>
+      </c>
+      <c r="C11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11">
+        <v>24</v>
+      </c>
+      <c r="F11" t="s">
+        <v>40</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
+      <c r="A12" s="1">
+        <v>46296.350347222222</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12">
+        <v>16</v>
+      </c>
+      <c r="F12" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
+      <c r="A13" s="1">
+        <v>46296.34447916667</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13">
+        <v>24</v>
+      </c>
+      <c r="F13" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
+      <c r="A14" s="1">
+        <v>46296.341724537036</v>
+      </c>
+      <c r="B14" s="1">
+        <v>46296.404004629629</v>
+      </c>
+      <c r="C14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
+      <c r="A15" s="1">
+        <v>46296.332986111112</v>
+      </c>
+      <c r="B15" s="1">
+        <v>46296.413587962961</v>
+      </c>
+      <c r="C15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15">
+        <v>24</v>
+      </c>
+      <c r="F15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="1"/>
-      <c r="B28" s="2"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
-      <c r="B29" s="2"/>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1"/>
+      <c r="A16" s="1">
+        <v>46296.330937500003</v>
+      </c>
+      <c r="B16" s="1">
+        <v>46296.400763888887</v>
+      </c>
+      <c r="C16" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16">
+        <v>16</v>
+      </c>
+      <c r="F16" t="s">
+        <v>58</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>46296.32234953704</v>
+      </c>
+      <c r="B17" s="1">
+        <v>46296.38863425926</v>
+      </c>
+      <c r="C17" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" t="s">
+        <v>61</v>
+      </c>
+      <c r="E17">
+        <v>16</v>
+      </c>
+      <c r="F17" t="s">
+        <v>62</v>
+      </c>
+      <c r="G17" t="s">
+        <v>63</v>
+      </c>
+      <c r="H17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>46296.318402777775</v>
+      </c>
+      <c r="B18" s="1">
+        <v>46296.394930555558</v>
+      </c>
+      <c r="C18" t="s">
+        <v>65</v>
+      </c>
+      <c r="D18" t="s">
+        <v>66</v>
+      </c>
+      <c r="E18">
+        <v>16</v>
+      </c>
+      <c r="F18" t="s">
+        <v>67</v>
+      </c>
+      <c r="G18" t="s">
+        <v>68</v>
+      </c>
+      <c r="H18" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>46296.309745370374</v>
+      </c>
+      <c r="B19" s="1">
+        <v>46296.411608796298</v>
+      </c>
+      <c r="C19" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" t="s">
+        <v>71</v>
+      </c>
+      <c r="E19">
+        <v>24</v>
+      </c>
+      <c r="F19" t="s">
+        <v>72</v>
+      </c>
+      <c r="G19" t="s">
+        <v>31</v>
+      </c>
+      <c r="H19" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>46296.306886574072</v>
+      </c>
+      <c r="B20" s="1">
+        <v>46296.361875000002</v>
+      </c>
+      <c r="C20" t="s">
+        <v>74</v>
+      </c>
+      <c r="D20" t="s">
+        <v>75</v>
+      </c>
+      <c r="E20">
+        <v>16</v>
+      </c>
+      <c r="F20" t="s">
+        <v>76</v>
+      </c>
+      <c r="G20" t="s">
+        <v>77</v>
+      </c>
+      <c r="H20" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>46296.305810185186</v>
+      </c>
+      <c r="B21" s="1">
+        <v>46296.38894675926</v>
+      </c>
+      <c r="C21" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21" t="s">
+        <v>80</v>
+      </c>
+      <c r="E21">
+        <v>8</v>
+      </c>
+      <c r="F21" t="s">
+        <v>81</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>46296.29855324074</v>
+      </c>
+      <c r="B22" s="1">
+        <v>46296.375752314816</v>
+      </c>
+      <c r="C22" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22">
+        <v>8</v>
+      </c>
+      <c r="F22" t="s">
+        <v>85</v>
+      </c>
+      <c r="G22" t="s">
+        <v>77</v>
+      </c>
+      <c r="H22" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>46296.297719907408</v>
+      </c>
+      <c r="B23" s="1">
+        <v>46296.370925925927</v>
+      </c>
+      <c r="C23" t="s">
+        <v>87</v>
+      </c>
+      <c r="D23" t="s">
+        <v>88</v>
+      </c>
+      <c r="E23">
+        <v>16</v>
+      </c>
+      <c r="F23" t="s">
+        <v>89</v>
+      </c>
+      <c r="G23" t="s">
+        <v>31</v>
+      </c>
+      <c r="H23" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>46296.294016203705</v>
+      </c>
+      <c r="B24" s="1">
+        <v>46296.395208333335</v>
+      </c>
+      <c r="C24" t="s">
+        <v>91</v>
+      </c>
+      <c r="D24" t="s">
+        <v>92</v>
+      </c>
+      <c r="E24">
+        <v>16</v>
+      </c>
+      <c r="F24" t="s">
+        <v>93</v>
+      </c>
+      <c r="G24" t="s">
+        <v>31</v>
+      </c>
+      <c r="H24" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>46296.290879629632</v>
+      </c>
+      <c r="B25" s="1">
+        <v>46296.375162037039</v>
+      </c>
+      <c r="C25" t="s">
+        <v>95</v>
+      </c>
+      <c r="D25" t="s">
+        <v>96</v>
+      </c>
+      <c r="E25">
+        <v>24</v>
+      </c>
+      <c r="F25" t="s">
+        <v>97</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>46296.287835648145</v>
+      </c>
+      <c r="B26" s="1">
+        <v>46296.40047453704</v>
+      </c>
+      <c r="C26" t="s">
+        <v>99</v>
+      </c>
+      <c r="D26" t="s">
+        <v>100</v>
+      </c>
+      <c r="E26">
+        <v>24</v>
+      </c>
+      <c r="F26" t="s">
+        <v>101</v>
+      </c>
+      <c r="G26" t="s">
+        <v>31</v>
+      </c>
+      <c r="H26" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>46296.286979166667</v>
+      </c>
+      <c r="B27" s="1">
+        <v>46296.382233796299</v>
+      </c>
+      <c r="C27" t="s">
+        <v>103</v>
+      </c>
+      <c r="D27" t="s">
+        <v>104</v>
+      </c>
+      <c r="E27">
+        <v>16</v>
+      </c>
+      <c r="F27" t="s">
+        <v>105</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>46296.28670138889</v>
+      </c>
+      <c r="B28" s="1">
+        <v>46296.381898148145</v>
+      </c>
+      <c r="C28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D28" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28">
+        <v>24</v>
+      </c>
+      <c r="F28" t="s">
+        <v>109</v>
+      </c>
+      <c r="G28" t="s">
+        <v>11</v>
+      </c>
+      <c r="H28" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>46296.283750000002</v>
+      </c>
+      <c r="B29" s="1">
+        <v>46296.351238425923</v>
+      </c>
+      <c r="C29" t="s">
+        <v>111</v>
+      </c>
+      <c r="D29" t="s">
+        <v>112</v>
+      </c>
+      <c r="E29">
+        <v>16</v>
+      </c>
+      <c r="F29" t="s">
+        <v>113</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>46296.282511574071</v>
+      </c>
+      <c r="B30" s="1">
+        <v>46296.346076388887</v>
+      </c>
+      <c r="C30" t="s">
+        <v>115</v>
+      </c>
+      <c r="D30" t="s">
+        <v>116</v>
+      </c>
+      <c r="E30">
+        <v>16</v>
+      </c>
+      <c r="F30" t="s">
+        <v>117</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>46296.272187499999</v>
+      </c>
+      <c r="B31" s="1">
+        <v>46296.340312499997</v>
+      </c>
+      <c r="C31" t="s">
+        <v>119</v>
+      </c>
+      <c r="D31" t="s">
+        <v>120</v>
+      </c>
+      <c r="E31">
+        <v>24</v>
+      </c>
+      <c r="F31" t="s">
+        <v>121</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>46296.270578703705</v>
+      </c>
+      <c r="B32" s="1">
+        <v>46296.369039351855</v>
+      </c>
+      <c r="C32" t="s">
+        <v>123</v>
+      </c>
+      <c r="D32" t="s">
+        <v>124</v>
+      </c>
+      <c r="E32">
+        <v>16</v>
+      </c>
+      <c r="F32" t="s">
+        <v>125</v>
+      </c>
+      <c r="G32" t="s">
+        <v>31</v>
+      </c>
+      <c r="H32" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
@@ -782,7 +1571,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="2"/>
+      <c r="B38" s="1"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
@@ -794,7 +1583,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="2"/>
+      <c r="B41" s="1"/>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
@@ -806,71 +1595,11 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
-      <c r="B44" s="2"/>
+      <c r="B44" s="1"/>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="1"/>
-      <c r="B46" s="1"/>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="1"/>
-      <c r="B47" s="1"/>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="1"/>
-      <c r="B48" s="1"/>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="1"/>
-      <c r="B50" s="1"/>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" s="1"/>
-      <c r="B52" s="1"/>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="1"/>
-      <c r="B53" s="1"/>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="1"/>
-      <c r="B54" s="1"/>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" s="1"/>
-      <c r="B55" s="1"/>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" s="1"/>
-      <c r="B56" s="2"/>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="1"/>
-      <c r="B57" s="1"/>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" s="1"/>
-      <c r="B58" s="1"/>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" s="1"/>
-      <c r="B59" s="1"/>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="1"/>
-      <c r="B60" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>